<commit_message>
refactor(tax): extract taxCalculationRealization into focused methods
- Extract logging logic into logCalculationStart() and logCalculationEnd()
- Extract tax rate calculation into calculateTaxRates() method
- Extract base tax calculation logic into calculateBaseTax() method
- Extract tax shield application into applyTaxShieldAndFinalize() method
- Simplify main taxCalculationRealization() method to orchestrate the flow
- Improve code maintainability and readability following SRP
- All 289 tests passing with 1201 assertions
</commit_message>
<xml_diff>
--- a/tests/Feature/config/salary_tenpercent.xlsx
+++ b/tests/Feature/config/salary_tenpercent.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="V6" s="3"/>
       <c r="W6" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X6" s="3"/>
       <c r="Y6" s="6">
@@ -1131,11 +1131,11 @@
       </c>
       <c r="V7" s="10"/>
       <c r="W7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X7" s="10"/>
       <c r="Y7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z7" s="11"/>
       <c r="AA7" s="9">
@@ -1234,11 +1234,11 @@
       </c>
       <c r="V8" s="3"/>
       <c r="W8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X8" s="3"/>
       <c r="Y8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z8" s="4"/>
       <c r="AA8" s="2">
@@ -1337,11 +1337,11 @@
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z9" s="4"/>
       <c r="AA9" s="2">
@@ -1440,11 +1440,11 @@
       </c>
       <c r="V10" s="3"/>
       <c r="W10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X10" s="3"/>
       <c r="Y10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z10" s="4"/>
       <c r="AA10" s="2">
@@ -1543,11 +1543,11 @@
       </c>
       <c r="V11" s="3"/>
       <c r="W11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z11" s="4"/>
       <c r="AA11" s="2">
@@ -1646,11 +1646,11 @@
       </c>
       <c r="V12" s="3"/>
       <c r="W12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X12" s="3"/>
       <c r="Y12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z12" s="4"/>
       <c r="AA12" s="2">
@@ -1749,11 +1749,11 @@
       </c>
       <c r="V13" s="3"/>
       <c r="W13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X13" s="3"/>
       <c r="Y13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z13" s="4"/>
       <c r="AA13" s="2">
@@ -1852,11 +1852,11 @@
       </c>
       <c r="V14" s="3"/>
       <c r="W14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X14" s="3"/>
       <c r="Y14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z14" s="4"/>
       <c r="AA14" s="2">
@@ -1955,11 +1955,11 @@
       </c>
       <c r="V15" s="3"/>
       <c r="W15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X15" s="3"/>
       <c r="Y15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z15" s="4"/>
       <c r="AA15" s="2">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="V16" s="3"/>
       <c r="W16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X16" s="3"/>
       <c r="Y16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z16" s="4"/>
       <c r="AA16" s="2">
@@ -2161,11 +2161,11 @@
       </c>
       <c r="V17" s="3"/>
       <c r="W17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X17" s="3"/>
       <c r="Y17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z17" s="4"/>
       <c r="AA17" s="2">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="V18" s="3"/>
       <c r="W18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X18" s="3"/>
       <c r="Y18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z18" s="4"/>
       <c r="AA18" s="2">
@@ -2367,11 +2367,11 @@
       </c>
       <c r="V19" s="3"/>
       <c r="W19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X19" s="3"/>
       <c r="Y19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z19" s="4"/>
       <c r="AA19" s="2">
@@ -2470,11 +2470,11 @@
       </c>
       <c r="V20" s="3"/>
       <c r="W20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X20" s="3"/>
       <c r="Y20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z20" s="4"/>
       <c r="AA20" s="2">
@@ -2573,11 +2573,11 @@
       </c>
       <c r="V21" s="3"/>
       <c r="W21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X21" s="3"/>
       <c r="Y21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z21" s="4"/>
       <c r="AA21" s="2">
@@ -2676,11 +2676,11 @@
       </c>
       <c r="V22" s="14"/>
       <c r="W22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X22" s="14"/>
       <c r="Y22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z22" s="15"/>
       <c r="AA22" s="13">
@@ -2779,11 +2779,11 @@
       </c>
       <c r="V23" s="3"/>
       <c r="W23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X23" s="3"/>
       <c r="Y23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z23" s="4"/>
       <c r="AA23" s="2">
@@ -2882,11 +2882,11 @@
       </c>
       <c r="V24" s="3"/>
       <c r="W24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X24" s="3"/>
       <c r="Y24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z24" s="4"/>
       <c r="AA24" s="2">
@@ -2985,11 +2985,11 @@
       </c>
       <c r="V25" s="3"/>
       <c r="W25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X25" s="3"/>
       <c r="Y25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z25" s="4"/>
       <c r="AA25" s="2">
@@ -3088,11 +3088,11 @@
       </c>
       <c r="V26" s="3"/>
       <c r="W26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X26" s="3"/>
       <c r="Y26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z26" s="4"/>
       <c r="AA26" s="2">
@@ -3191,11 +3191,11 @@
       </c>
       <c r="V27" s="3"/>
       <c r="W27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X27" s="3"/>
       <c r="Y27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z27" s="4"/>
       <c r="AA27" s="2">
@@ -3294,11 +3294,11 @@
       </c>
       <c r="V28" s="3"/>
       <c r="W28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X28" s="3"/>
       <c r="Y28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z28" s="4"/>
       <c r="AA28" s="2">
@@ -3397,11 +3397,11 @@
       </c>
       <c r="V29" s="3"/>
       <c r="W29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z29" s="4"/>
       <c r="AA29" s="2">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="V30" s="18"/>
       <c r="W30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X30" s="18"/>
       <c r="Y30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z30" s="19"/>
       <c r="AA30" s="17">
@@ -3603,11 +3603,11 @@
       </c>
       <c r="V31" s="3"/>
       <c r="W31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X31" s="3"/>
       <c r="Y31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z31" s="4"/>
       <c r="AA31" s="2">
@@ -3706,11 +3706,11 @@
       </c>
       <c r="V32" s="3"/>
       <c r="W32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X32" s="3"/>
       <c r="Y32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z32" s="4"/>
       <c r="AA32" s="2">
@@ -3809,11 +3809,11 @@
       </c>
       <c r="V33" s="3"/>
       <c r="W33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X33" s="3"/>
       <c r="Y33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z33" s="4"/>
       <c r="AA33" s="2">
@@ -3912,11 +3912,11 @@
       </c>
       <c r="V34" s="18"/>
       <c r="W34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X34" s="18"/>
       <c r="Y34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z34" s="19"/>
       <c r="AA34" s="17">
@@ -4015,11 +4015,11 @@
       </c>
       <c r="V35" s="3"/>
       <c r="W35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X35" s="3"/>
       <c r="Y35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z35" s="4"/>
       <c r="AA35" s="2">
@@ -4118,11 +4118,11 @@
       </c>
       <c r="V36" s="3"/>
       <c r="W36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X36" s="3"/>
       <c r="Y36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z36" s="4"/>
       <c r="AA36" s="2">
@@ -4221,11 +4221,11 @@
       </c>
       <c r="V37" s="3"/>
       <c r="W37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X37" s="3"/>
       <c r="Y37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z37" s="4"/>
       <c r="AA37" s="2">
@@ -4324,11 +4324,11 @@
       </c>
       <c r="V38" s="3"/>
       <c r="W38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X38" s="3"/>
       <c r="Y38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z38" s="4"/>
       <c r="AA38" s="2">
@@ -4427,11 +4427,11 @@
       </c>
       <c r="V39" s="3"/>
       <c r="W39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X39" s="3"/>
       <c r="Y39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z39" s="4"/>
       <c r="AA39" s="2">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="V6" s="3"/>
       <c r="W6" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X6" s="3"/>
       <c r="Y6" s="6">
@@ -5027,11 +5027,11 @@
       </c>
       <c r="V7" s="10"/>
       <c r="W7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X7" s="10"/>
       <c r="Y7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z7" s="11"/>
       <c r="AA7" s="9">
@@ -5130,11 +5130,11 @@
       </c>
       <c r="V8" s="3"/>
       <c r="W8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X8" s="3"/>
       <c r="Y8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z8" s="4"/>
       <c r="AA8" s="2">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z9" s="4"/>
       <c r="AA9" s="2">
@@ -5336,11 +5336,11 @@
       </c>
       <c r="V10" s="3"/>
       <c r="W10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X10" s="3"/>
       <c r="Y10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z10" s="4"/>
       <c r="AA10" s="2">
@@ -5439,11 +5439,11 @@
       </c>
       <c r="V11" s="3"/>
       <c r="W11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z11" s="4"/>
       <c r="AA11" s="2">
@@ -5542,11 +5542,11 @@
       </c>
       <c r="V12" s="3"/>
       <c r="W12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X12" s="3"/>
       <c r="Y12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z12" s="4"/>
       <c r="AA12" s="2">
@@ -5645,11 +5645,11 @@
       </c>
       <c r="V13" s="3"/>
       <c r="W13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X13" s="3"/>
       <c r="Y13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z13" s="4"/>
       <c r="AA13" s="2">
@@ -5748,11 +5748,11 @@
       </c>
       <c r="V14" s="3"/>
       <c r="W14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X14" s="3"/>
       <c r="Y14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z14" s="4"/>
       <c r="AA14" s="2">
@@ -5851,11 +5851,11 @@
       </c>
       <c r="V15" s="3"/>
       <c r="W15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X15" s="3"/>
       <c r="Y15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z15" s="4"/>
       <c r="AA15" s="2">
@@ -5954,11 +5954,11 @@
       </c>
       <c r="V16" s="3"/>
       <c r="W16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X16" s="3"/>
       <c r="Y16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z16" s="4"/>
       <c r="AA16" s="2">
@@ -6057,11 +6057,11 @@
       </c>
       <c r="V17" s="3"/>
       <c r="W17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X17" s="3"/>
       <c r="Y17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z17" s="4"/>
       <c r="AA17" s="2">
@@ -6160,11 +6160,11 @@
       </c>
       <c r="V18" s="3"/>
       <c r="W18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X18" s="3"/>
       <c r="Y18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z18" s="4"/>
       <c r="AA18" s="2">
@@ -6263,11 +6263,11 @@
       </c>
       <c r="V19" s="3"/>
       <c r="W19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X19" s="3"/>
       <c r="Y19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z19" s="4"/>
       <c r="AA19" s="2">
@@ -6366,11 +6366,11 @@
       </c>
       <c r="V20" s="3"/>
       <c r="W20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X20" s="3"/>
       <c r="Y20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z20" s="4"/>
       <c r="AA20" s="2">
@@ -6469,11 +6469,11 @@
       </c>
       <c r="V21" s="3"/>
       <c r="W21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X21" s="3"/>
       <c r="Y21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z21" s="4"/>
       <c r="AA21" s="2">
@@ -6572,11 +6572,11 @@
       </c>
       <c r="V22" s="14"/>
       <c r="W22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X22" s="14"/>
       <c r="Y22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z22" s="15"/>
       <c r="AA22" s="13">
@@ -6675,11 +6675,11 @@
       </c>
       <c r="V23" s="3"/>
       <c r="W23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X23" s="3"/>
       <c r="Y23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z23" s="4"/>
       <c r="AA23" s="2">
@@ -6778,11 +6778,11 @@
       </c>
       <c r="V24" s="3"/>
       <c r="W24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X24" s="3"/>
       <c r="Y24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z24" s="4"/>
       <c r="AA24" s="2">
@@ -6881,11 +6881,11 @@
       </c>
       <c r="V25" s="3"/>
       <c r="W25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X25" s="3"/>
       <c r="Y25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z25" s="4"/>
       <c r="AA25" s="2">
@@ -6984,11 +6984,11 @@
       </c>
       <c r="V26" s="3"/>
       <c r="W26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X26" s="3"/>
       <c r="Y26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z26" s="4"/>
       <c r="AA26" s="2">
@@ -7087,11 +7087,11 @@
       </c>
       <c r="V27" s="3"/>
       <c r="W27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X27" s="3"/>
       <c r="Y27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z27" s="4"/>
       <c r="AA27" s="2">
@@ -7190,11 +7190,11 @@
       </c>
       <c r="V28" s="3"/>
       <c r="W28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X28" s="3"/>
       <c r="Y28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z28" s="4"/>
       <c r="AA28" s="2">
@@ -7293,11 +7293,11 @@
       </c>
       <c r="V29" s="3"/>
       <c r="W29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z29" s="4"/>
       <c r="AA29" s="2">
@@ -7396,11 +7396,11 @@
       </c>
       <c r="V30" s="18"/>
       <c r="W30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X30" s="18"/>
       <c r="Y30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z30" s="19"/>
       <c r="AA30" s="17">
@@ -7499,11 +7499,11 @@
       </c>
       <c r="V31" s="3"/>
       <c r="W31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X31" s="3"/>
       <c r="Y31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z31" s="4"/>
       <c r="AA31" s="2">
@@ -7602,11 +7602,11 @@
       </c>
       <c r="V32" s="3"/>
       <c r="W32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X32" s="3"/>
       <c r="Y32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z32" s="4"/>
       <c r="AA32" s="2">
@@ -7705,11 +7705,11 @@
       </c>
       <c r="V33" s="3"/>
       <c r="W33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X33" s="3"/>
       <c r="Y33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z33" s="4"/>
       <c r="AA33" s="2">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="V34" s="18"/>
       <c r="W34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X34" s="18"/>
       <c r="Y34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z34" s="19"/>
       <c r="AA34" s="17">
@@ -7911,11 +7911,11 @@
       </c>
       <c r="V35" s="3"/>
       <c r="W35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X35" s="3"/>
       <c r="Y35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z35" s="4"/>
       <c r="AA35" s="2">
@@ -8014,11 +8014,11 @@
       </c>
       <c r="V36" s="3"/>
       <c r="W36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X36" s="3"/>
       <c r="Y36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z36" s="4"/>
       <c r="AA36" s="2">
@@ -8117,11 +8117,11 @@
       </c>
       <c r="V37" s="3"/>
       <c r="W37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X37" s="3"/>
       <c r="Y37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z37" s="4"/>
       <c r="AA37" s="2">
@@ -8220,11 +8220,11 @@
       </c>
       <c r="V38" s="3"/>
       <c r="W38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X38" s="3"/>
       <c r="Y38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z38" s="4"/>
       <c r="AA38" s="2">
@@ -8323,11 +8323,11 @@
       </c>
       <c r="V39" s="3"/>
       <c r="W39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X39" s="3"/>
       <c r="Y39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z39" s="4"/>
       <c r="AA39" s="2">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="V6" s="3"/>
       <c r="W6" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X6" s="3"/>
       <c r="Y6" s="6"/>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="V7" s="10"/>
       <c r="W7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X7" s="10"/>
       <c r="Y7" s="9"/>
@@ -8912,7 +8912,7 @@
       </c>
       <c r="V8" s="3"/>
       <c r="W8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X8" s="3"/>
       <c r="Y8" s="6"/>
@@ -8969,7 +8969,7 @@
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="6"/>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="V10" s="3"/>
       <c r="W10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X10" s="3"/>
       <c r="Y10" s="6"/>
@@ -9083,7 +9083,7 @@
       </c>
       <c r="V11" s="3"/>
       <c r="W11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="6"/>
@@ -9140,7 +9140,7 @@
       </c>
       <c r="V12" s="3"/>
       <c r="W12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X12" s="3"/>
       <c r="Y12" s="6"/>
@@ -9197,7 +9197,7 @@
       </c>
       <c r="V13" s="3"/>
       <c r="W13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X13" s="3"/>
       <c r="Y13" s="6"/>
@@ -9254,7 +9254,7 @@
       </c>
       <c r="V14" s="3"/>
       <c r="W14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X14" s="3"/>
       <c r="Y14" s="6"/>
@@ -9311,7 +9311,7 @@
       </c>
       <c r="V15" s="3"/>
       <c r="W15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X15" s="3"/>
       <c r="Y15" s="6"/>
@@ -9368,7 +9368,7 @@
       </c>
       <c r="V16" s="3"/>
       <c r="W16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X16" s="3"/>
       <c r="Y16" s="6"/>
@@ -9425,7 +9425,7 @@
       </c>
       <c r="V17" s="3"/>
       <c r="W17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X17" s="3"/>
       <c r="Y17" s="6"/>
@@ -9482,7 +9482,7 @@
       </c>
       <c r="V18" s="3"/>
       <c r="W18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X18" s="3"/>
       <c r="Y18" s="6"/>
@@ -9539,7 +9539,7 @@
       </c>
       <c r="V19" s="3"/>
       <c r="W19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X19" s="3"/>
       <c r="Y19" s="6"/>
@@ -9596,7 +9596,7 @@
       </c>
       <c r="V20" s="3"/>
       <c r="W20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X20" s="3"/>
       <c r="Y20" s="6"/>
@@ -9653,7 +9653,7 @@
       </c>
       <c r="V21" s="3"/>
       <c r="W21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X21" s="3"/>
       <c r="Y21" s="6"/>
@@ -9710,7 +9710,7 @@
       </c>
       <c r="V22" s="14"/>
       <c r="W22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X22" s="14"/>
       <c r="Y22" s="13"/>
@@ -9767,7 +9767,7 @@
       </c>
       <c r="V23" s="3"/>
       <c r="W23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X23" s="3"/>
       <c r="Y23" s="6"/>
@@ -9824,7 +9824,7 @@
       </c>
       <c r="V24" s="3"/>
       <c r="W24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X24" s="3"/>
       <c r="Y24" s="6"/>
@@ -9881,7 +9881,7 @@
       </c>
       <c r="V25" s="3"/>
       <c r="W25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X25" s="3"/>
       <c r="Y25" s="6"/>
@@ -9938,7 +9938,7 @@
       </c>
       <c r="V26" s="3"/>
       <c r="W26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X26" s="3"/>
       <c r="Y26" s="6"/>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="V27" s="3"/>
       <c r="W27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X27" s="3"/>
       <c r="Y27" s="6"/>
@@ -10052,7 +10052,7 @@
       </c>
       <c r="V28" s="3"/>
       <c r="W28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X28" s="3"/>
       <c r="Y28" s="6"/>
@@ -10109,7 +10109,7 @@
       </c>
       <c r="V29" s="3"/>
       <c r="W29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="6"/>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="V30" s="18"/>
       <c r="W30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X30" s="18"/>
       <c r="Y30" s="17"/>
@@ -10223,7 +10223,7 @@
       </c>
       <c r="V31" s="3"/>
       <c r="W31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X31" s="3"/>
       <c r="Y31" s="6"/>
@@ -10280,7 +10280,7 @@
       </c>
       <c r="V32" s="3"/>
       <c r="W32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X32" s="3"/>
       <c r="Y32" s="6"/>
@@ -10337,7 +10337,7 @@
       </c>
       <c r="V33" s="3"/>
       <c r="W33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X33" s="3"/>
       <c r="Y33" s="6"/>
@@ -10394,7 +10394,7 @@
       </c>
       <c r="V34" s="18"/>
       <c r="W34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X34" s="18"/>
       <c r="Y34" s="17"/>
@@ -10451,7 +10451,7 @@
       </c>
       <c r="V35" s="3"/>
       <c r="W35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X35" s="3"/>
       <c r="Y35" s="6"/>
@@ -10508,7 +10508,7 @@
       </c>
       <c r="V36" s="3"/>
       <c r="W36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X36" s="3"/>
       <c r="Y36" s="6"/>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="V37" s="3"/>
       <c r="W37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X37" s="3"/>
       <c r="Y37" s="6"/>
@@ -10622,7 +10622,7 @@
       </c>
       <c r="V38" s="3"/>
       <c r="W38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X38" s="3"/>
       <c r="Y38" s="6"/>
@@ -10679,7 +10679,7 @@
       </c>
       <c r="V39" s="3"/>
       <c r="W39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X39" s="3"/>
       <c r="Y39" s="6"/>
@@ -11153,13 +11153,9 @@
         <v>0</v>
       </c>
       <c r="V6" s="3"/>
-      <c r="W6" s="6">
-        <v>0</v>
-      </c>
+      <c r="W6" s="6"/>
       <c r="X6" s="3"/>
-      <c r="Y6" s="6">
-        <v>0</v>
-      </c>
+      <c r="Y6" s="6"/>
       <c r="Z6" s="4"/>
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
@@ -11239,11 +11235,11 @@
       </c>
       <c r="V7" s="10"/>
       <c r="W7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X7" s="10"/>
       <c r="Y7" s="9">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z7" s="11"/>
       <c r="AA7" s="9"/>
@@ -11326,11 +11322,11 @@
       </c>
       <c r="V8" s="3"/>
       <c r="W8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X8" s="3"/>
       <c r="Y8" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z8" s="4"/>
       <c r="AA8" s="2"/>
@@ -11413,11 +11409,11 @@
       </c>
       <c r="V9" s="3"/>
       <c r="W9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X9" s="3"/>
       <c r="Y9" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z9" s="4"/>
       <c r="AA9" s="2"/>
@@ -11500,11 +11496,11 @@
       </c>
       <c r="V10" s="3"/>
       <c r="W10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X10" s="3"/>
       <c r="Y10" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z10" s="4"/>
       <c r="AA10" s="2"/>
@@ -11587,11 +11583,11 @@
       </c>
       <c r="V11" s="3"/>
       <c r="W11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X11" s="3"/>
       <c r="Y11" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z11" s="4"/>
       <c r="AA11" s="2"/>
@@ -11674,11 +11670,11 @@
       </c>
       <c r="V12" s="3"/>
       <c r="W12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X12" s="3"/>
       <c r="Y12" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z12" s="4"/>
       <c r="AA12" s="2"/>
@@ -11761,11 +11757,11 @@
       </c>
       <c r="V13" s="3"/>
       <c r="W13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X13" s="3"/>
       <c r="Y13" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z13" s="4"/>
       <c r="AA13" s="2"/>
@@ -11848,11 +11844,11 @@
       </c>
       <c r="V14" s="3"/>
       <c r="W14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X14" s="3"/>
       <c r="Y14" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z14" s="4"/>
       <c r="AA14" s="2"/>
@@ -11935,11 +11931,11 @@
       </c>
       <c r="V15" s="3"/>
       <c r="W15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X15" s="3"/>
       <c r="Y15" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z15" s="4"/>
       <c r="AA15" s="2"/>
@@ -12022,11 +12018,11 @@
       </c>
       <c r="V16" s="3"/>
       <c r="W16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X16" s="3"/>
       <c r="Y16" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z16" s="4"/>
       <c r="AA16" s="2"/>
@@ -12109,11 +12105,11 @@
       </c>
       <c r="V17" s="3"/>
       <c r="W17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X17" s="3"/>
       <c r="Y17" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z17" s="4"/>
       <c r="AA17" s="2"/>
@@ -12196,11 +12192,11 @@
       </c>
       <c r="V18" s="3"/>
       <c r="W18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X18" s="3"/>
       <c r="Y18" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z18" s="4"/>
       <c r="AA18" s="2"/>
@@ -12283,11 +12279,11 @@
       </c>
       <c r="V19" s="3"/>
       <c r="W19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X19" s="3"/>
       <c r="Y19" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z19" s="4"/>
       <c r="AA19" s="2"/>
@@ -12370,11 +12366,11 @@
       </c>
       <c r="V20" s="3"/>
       <c r="W20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X20" s="3"/>
       <c r="Y20" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z20" s="4"/>
       <c r="AA20" s="2"/>
@@ -12457,11 +12453,11 @@
       </c>
       <c r="V21" s="3"/>
       <c r="W21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X21" s="3"/>
       <c r="Y21" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z21" s="4"/>
       <c r="AA21" s="2"/>
@@ -12544,11 +12540,11 @@
       </c>
       <c r="V22" s="14"/>
       <c r="W22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X22" s="14"/>
       <c r="Y22" s="13">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z22" s="15"/>
       <c r="AA22" s="13"/>
@@ -12631,11 +12627,11 @@
       </c>
       <c r="V23" s="3"/>
       <c r="W23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X23" s="3"/>
       <c r="Y23" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z23" s="4"/>
       <c r="AA23" s="2"/>
@@ -12718,11 +12714,11 @@
       </c>
       <c r="V24" s="3"/>
       <c r="W24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X24" s="3"/>
       <c r="Y24" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z24" s="4"/>
       <c r="AA24" s="2"/>
@@ -12805,11 +12801,11 @@
       </c>
       <c r="V25" s="3"/>
       <c r="W25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X25" s="3"/>
       <c r="Y25" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z25" s="4"/>
       <c r="AA25" s="2"/>
@@ -12892,11 +12888,11 @@
       </c>
       <c r="V26" s="3"/>
       <c r="W26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X26" s="3"/>
       <c r="Y26" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z26" s="4"/>
       <c r="AA26" s="2"/>
@@ -12979,11 +12975,11 @@
       </c>
       <c r="V27" s="3"/>
       <c r="W27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X27" s="3"/>
       <c r="Y27" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z27" s="4"/>
       <c r="AA27" s="2"/>
@@ -13066,11 +13062,11 @@
       </c>
       <c r="V28" s="3"/>
       <c r="W28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X28" s="3"/>
       <c r="Y28" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z28" s="4"/>
       <c r="AA28" s="2"/>
@@ -13153,11 +13149,11 @@
       </c>
       <c r="V29" s="3"/>
       <c r="W29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z29" s="4"/>
       <c r="AA29" s="2"/>
@@ -13240,11 +13236,11 @@
       </c>
       <c r="V30" s="18"/>
       <c r="W30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X30" s="18"/>
       <c r="Y30" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z30" s="19"/>
       <c r="AA30" s="17"/>
@@ -13327,11 +13323,11 @@
       </c>
       <c r="V31" s="3"/>
       <c r="W31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X31" s="3"/>
       <c r="Y31" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z31" s="4"/>
       <c r="AA31" s="2"/>
@@ -13414,11 +13410,11 @@
       </c>
       <c r="V32" s="3"/>
       <c r="W32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X32" s="3"/>
       <c r="Y32" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z32" s="4"/>
       <c r="AA32" s="2"/>
@@ -13501,11 +13497,11 @@
       </c>
       <c r="V33" s="3"/>
       <c r="W33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X33" s="3"/>
       <c r="Y33" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z33" s="4"/>
       <c r="AA33" s="2"/>
@@ -13588,11 +13584,11 @@
       </c>
       <c r="V34" s="18"/>
       <c r="W34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X34" s="18"/>
       <c r="Y34" s="17">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z34" s="19"/>
       <c r="AA34" s="17"/>
@@ -13675,11 +13671,11 @@
       </c>
       <c r="V35" s="3"/>
       <c r="W35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X35" s="3"/>
       <c r="Y35" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z35" s="4"/>
       <c r="AA35" s="2"/>
@@ -13762,11 +13758,11 @@
       </c>
       <c r="V36" s="3"/>
       <c r="W36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X36" s="3"/>
       <c r="Y36" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z36" s="4"/>
       <c r="AA36" s="2"/>
@@ -13849,11 +13845,11 @@
       </c>
       <c r="V37" s="3"/>
       <c r="W37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X37" s="3"/>
       <c r="Y37" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z37" s="4"/>
       <c r="AA37" s="2"/>
@@ -13936,11 +13932,11 @@
       </c>
       <c r="V38" s="3"/>
       <c r="W38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X38" s="3"/>
       <c r="Y38" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z38" s="4"/>
       <c r="AA38" s="2"/>
@@ -14023,11 +14019,11 @@
       </c>
       <c r="V39" s="3"/>
       <c r="W39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="X39" s="3"/>
       <c r="Y39" s="6">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="Z39" s="4"/>
       <c r="AA39" s="2"/>
@@ -14209,9 +14205,295 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <sheetData>
+    <row r="6" spans="1:1">
+      <c r="A6">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34">
+        <v>2029</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37">
+        <v>2032</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38">
+        <v>2033</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41">
+        <v>2036</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42">
+        <v>2037</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43">
+        <v>2038</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44">
+        <v>2039</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48">
+        <v>2043</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49">
+        <v>2044</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50">
+        <v>2045</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51">
+        <v>2046</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52">
+        <v>2047</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54">
+        <v>2049</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56">
+        <v>2051</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59">
+        <v>2054</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61">
+        <v>2056</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62">
+        <v>2057</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>

</xml_diff>